<commit_message>
docs: facturación con dos razones sociales (AGROMORALES / CEBALLOS Y LOZANO)
- Skill managing-facturacion al día: estado real (código en main, menú oculto,
  27 tarifas de ejemplo), la razón social como parte de la llave de la tarifa,
  Riopaila Agrícola ≠ Ingenio Riopaila, el cruce tabla × realizado y la plantilla.
- Plantilla: pregunta la fecha desde la que se FACTURA desde la app (no facturar
  hacia atrás, decisión de agosto), el programa de facturación y los datos de
  cada cliente.
- CLAUDE.md: filas de Tarifas y Fincas (varias pasadas, quién reporta).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
+++ b/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
@@ -29016,7 +29016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -29069,12 +29069,12 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Para valorar lo ya hecho desde mayo con el precio que tocaba en su fecha.</t>
+          <t>Para valorar lo ya hecho con el precio que tocaba en su fecha.</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Desde el 16-may-2026 (primera labor en la app)</t>
+          <t>Desde el 16-may-2026 (primera labor en la app), solo para ver el valor</t>
         </is>
       </c>
       <c r="D5" s="11" t="n"/>
@@ -29082,17 +29082,17 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>¿Los precios incluyen IVA? ¿Qué impuestos o retenciones lleva la factura?</t>
+          <t>¿Desde qué fecha se empieza a FACTURAR desde la app? Lo anterior ya se facturó por fuera.</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Para que el total de la pre-factura cuadre con la factura real.</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Precio antes de IVA; la app muestra IVA aparte</t>
+          <t>Para no volver a cobrar lo que ya se facturó: antes de esa fecha la app solo muestra el valor, no arma cobro.</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Desde el 1-oct-2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="n"/>
@@ -29100,17 +29100,17 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>¿Cada cuánto se factura: quincenal o mensual? ¿Por cliente o por hacienda?</t>
+          <t>¿En qué programa emiten hoy la factura electrónica (Siigo u otro)? ¿Quién la emite?</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Así se agrupan las líneas en cada pre-factura.</t>
+          <t>El número legal y el envío a la DIAN salen de ese programa; la app arma la cuenta de cobro y la pre-factura.</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Quincenal, una por razón social + cliente</t>
+          <t>La app entrega la pre-factura; el número lo da el programa de facturación</t>
         </is>
       </c>
       <c r="D7" s="11" t="n"/>
@@ -29118,17 +29118,17 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>¿Se factura el área REALIZADA (la que reporta el operador) o el área de la suerte (maestro)?</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Cambia el valor de cada línea.</t>
+          <t>Datos de cada cliente para facturar: razón social, NIT y correo de facturación.</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Para que la pre-factura salga completa por cliente.</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Área realizada, como en la planilla</t>
+          <t>Los traen las facturas de ejemplo</t>
         </is>
       </c>
       <c r="D8" s="11" t="n"/>
@@ -29136,17 +29136,17 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>¿El ingenio pide número de orden de servicio / OT / pedido en cada línea?</t>
+          <t>¿Los precios incluyen IVA? ¿Qué impuestos o retenciones lleva la factura?</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Si lo exige, la app debe pedirlo al asignar.</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Campo opcional por labor</t>
+          <t>Para que el total de la pre-factura cuadre con la factura real.</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Precio antes de IVA; la app muestra IVA aparte</t>
         </is>
       </c>
       <c r="D9" s="11" t="n"/>
@@ -29154,17 +29154,17 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>¿Quién aprueba antes de facturar? ¿Se factura solo lo aprobado?</t>
+          <t>¿Cada cuánto se factura: quincenal o mensual? ¿Por cliente o por hacienda?</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Evita facturar labores sin revisar.</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Solo labores aprobadas</t>
+          <t>Así se agrupan las líneas en cada pre-factura.</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Quincenal, una por razón social + cliente</t>
         </is>
       </c>
       <c r="D10" s="11" t="n"/>
@@ -29172,17 +29172,17 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>¿Hay reajuste anual de tarifas? ¿En qué fecha y cómo (IPC, %)?</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>La app guarda cada precio con su vigencia; el cambio no toca lo ya facturado.</t>
+          <t>¿Se factura el área REALIZADA (la que reporta el operador) o el área de la suerte (maestro)?</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Cambia el valor de cada línea.</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Se carga el precio nuevo con su fecha</t>
+          <t>Área realizada, como en la planilla</t>
         </is>
       </c>
       <c r="D11" s="11" t="n"/>
@@ -29190,34 +29190,88 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>¿Quién de ustedes es el contacto para dudas de precios?</t>
+          <t>¿El ingenio pide número de orden de servicio / OT / pedido en cada línea?</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Para resolver rápido las líneas «sin tarifa».</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr"/>
+          <t>Si lo exige, la app debe pedirlo al asignar.</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Campo opcional por labor</t>
+        </is>
+      </c>
       <c r="D12" s="11" t="n"/>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
+          <t>¿Quién aprueba antes de facturar? ¿Se factura solo lo aprobado?</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Evita facturar labores sin revisar.</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Solo labores aprobadas</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>¿Hay reajuste anual de tarifas? ¿En qué fecha y cómo (IPC, %)?</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>La app guarda cada precio con su vigencia; el cambio no toca lo ya facturado.</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Se carga el precio nuevo con su fecha</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>¿Quién de ustedes es el contacto para dudas de precios?</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Para resolver rápido las líneas «sin tarifa».</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
           <t>¿Nos pueden pasar una factura ya emitida (de cada razón social) como ejemplo?</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Para que la pre-factura salga en el mismo formato y con los mismos datos.</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>Una de AGROMORALES y una de CEBALLOS Y LOZANO</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(facturación): modalidad de la labor en la skill, la guía y la plantilla
La plantilla del cliente pide ahora cada precio por «LABOR · MODALIDAD» y la hoja 5
confirma lo dudoso de la hoja escrita (triple, fertilización, cultivo, acequias por
pase o por hectómetro).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
+++ b/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
@@ -810,7 +810,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -824,7 +824,11 @@
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="13" t="n"/>
       <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="inlineStr"/>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -844,7 +848,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -858,7 +862,11 @@
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="13" t="n"/>
       <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -878,7 +886,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -892,7 +900,11 @@
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n"/>
       <c r="I7" s="11" t="n"/>
-      <c r="J7" s="11" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -912,7 +924,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -926,7 +938,11 @@
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="13" t="n"/>
       <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="inlineStr"/>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -946,7 +962,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE V</t>
+          <t>REENCALLE · VERDE</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -962,7 +978,7 @@
       <c r="I9" s="11" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Suponemos que la «REENCALLE V» de la app es este reencalle de caña verde/cruda: confirmar</t>
+          <t>Reencalle modalidad VERDE (caña verde / cruda): confirmar</t>
         </is>
       </c>
     </row>
@@ -984,7 +1000,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>TRIPLE</t>
+          <t>TRIPLE · TODAS</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -998,7 +1014,11 @@
       <c r="G10" s="11" t="n"/>
       <c r="H10" s="13" t="n"/>
       <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="inlineStr"/>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1018,7 +1038,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>CULTIVO</t>
+          <t>CULTIVO · TODAS</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -1032,7 +1052,11 @@
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="inlineStr"/>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1052,7 +1076,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>OFICIOS VARIOS JORNAL (nueva)</t>
+          <t>OFICIOS VARIOS (jornal)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -1066,11 +1090,7 @@
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1090,7 +1110,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -1104,7 +1124,11 @@
       <c r="G13" s="11" t="n"/>
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1122,9 +1146,9 @@
           <t>Abono Plantilla</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>FERTILIZACION PLANTILLA (nueva)</t>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>FERTILIZACION · PLANTILLA</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -1138,11 +1162,7 @@
       <c r="G14" s="11" t="n"/>
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -1162,7 +1182,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>FERTILIZACION 2X1 (nueva)</t>
+          <t>FERTILIZACION · 2X1</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -1176,11 +1196,7 @@
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="11" t="n"/>
-      <c r="J15" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1200,7 +1216,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>FERTILIZACION 4X1 (nueva)</t>
+          <t>FERTILIZACION · 4X1</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -1214,11 +1230,7 @@
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="11" t="n"/>
-      <c r="J16" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -1236,11 +1248,7 @@
           <t>Acequias</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>ACEQUIAS</t>
-        </is>
-      </c>
+      <c r="D17" s="11" t="n"/>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="12" t="n">
         <v>70000</v>
@@ -1306,7 +1314,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>SUBSUELO</t>
+          <t>SUBSUELO · TODAS</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -1320,7 +1328,11 @@
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="13" t="n"/>
       <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="inlineStr"/>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -1340,7 +1352,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>TRIPLE</t>
+          <t>TRIPLE · TODAS</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -1354,7 +1366,11 @@
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="inlineStr"/>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -1374,7 +1390,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>CULTIVO</t>
+          <t>CULTIVO · TODAS</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1388,7 +1404,11 @@
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="13" t="n"/>
       <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="inlineStr"/>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -1408,7 +1428,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -1422,7 +1442,11 @@
       <c r="G22" s="11" t="n"/>
       <c r="H22" s="13" t="n"/>
       <c r="I22" s="11" t="n"/>
-      <c r="J22" s="11" t="inlineStr"/>
+      <c r="J22" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -1442,7 +1466,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -1456,7 +1480,11 @@
       <c r="G23" s="11" t="n"/>
       <c r="H23" s="13" t="n"/>
       <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="inlineStr"/>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -1476,7 +1504,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -1490,7 +1518,11 @@
       <c r="G24" s="11" t="n"/>
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="inlineStr"/>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -1510,7 +1542,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -1524,7 +1556,11 @@
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="inlineStr"/>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -1544,7 +1580,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -1558,7 +1594,11 @@
       <c r="G26" s="11" t="n"/>
       <c r="H26" s="13" t="n"/>
       <c r="I26" s="11" t="n"/>
-      <c r="J26" s="11" t="inlineStr"/>
+      <c r="J26" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -1578,7 +1618,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -1592,7 +1632,11 @@
       <c r="G27" s="11" t="n"/>
       <c r="H27" s="13" t="n"/>
       <c r="I27" s="11" t="n"/>
-      <c r="J27" s="11" t="inlineStr"/>
+      <c r="J27" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -1612,7 +1656,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>SUBSUELO</t>
+          <t>SUBSUELO · TODAS</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -1626,7 +1670,11 @@
       <c r="G28" s="11" t="n"/>
       <c r="H28" s="13" t="n"/>
       <c r="I28" s="11" t="n"/>
-      <c r="J28" s="11" t="inlineStr"/>
+      <c r="J28" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -1646,7 +1694,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>TRIPLE</t>
+          <t>TRIPLE · TODAS</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -1660,7 +1708,11 @@
       <c r="G29" s="11" t="n"/>
       <c r="H29" s="13" t="n"/>
       <c r="I29" s="11" t="n"/>
-      <c r="J29" s="11" t="inlineStr"/>
+      <c r="J29" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -1680,7 +1732,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -1694,7 +1746,11 @@
       <c r="G30" s="11" t="n"/>
       <c r="H30" s="13" t="n"/>
       <c r="I30" s="11" t="n"/>
-      <c r="J30" s="11" t="inlineStr"/>
+      <c r="J30" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -1714,7 +1770,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
@@ -1728,7 +1784,11 @@
       <c r="G31" s="11" t="n"/>
       <c r="H31" s="13" t="n"/>
       <c r="I31" s="11" t="n"/>
-      <c r="J31" s="11" t="inlineStr"/>
+      <c r="J31" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -1748,7 +1808,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>REENCALLE V</t>
+          <t>REENCALLE · VERDE</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -1764,7 +1824,7 @@
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>Suponemos que la «REENCALLE V» de la app es este reencalle de caña verde/cruda: confirmar</t>
+          <t>Reencalle modalidad VERDE (caña verde / cruda): confirmar</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1846,7 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>SUBSUELO</t>
+          <t>SUBSUELO · TODAS</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
@@ -1800,7 +1860,11 @@
       <c r="G33" s="11" t="n"/>
       <c r="H33" s="13" t="n"/>
       <c r="I33" s="11" t="n"/>
-      <c r="J33" s="11" t="inlineStr"/>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -1820,7 +1884,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>TRIPLE</t>
+          <t>TRIPLE · TODAS</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -1834,7 +1898,11 @@
       <c r="G34" s="11" t="n"/>
       <c r="H34" s="13" t="n"/>
       <c r="I34" s="11" t="n"/>
-      <c r="J34" s="11" t="inlineStr"/>
+      <c r="J34" s="14" t="inlineStr">
+        <is>
+          <t>¿Este precio vale para TODAS las modalidades? Si no, escoja la modalidad en la columna D y agregue abajo el precio de las otras</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -1854,7 +1922,7 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>SUBSUELO 4X1 (nueva)</t>
+          <t>SUBSUELO · 4X1</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -1868,11 +1936,7 @@
       <c r="G35" s="11" t="n"/>
       <c r="H35" s="13" t="n"/>
       <c r="I35" s="11" t="n"/>
-      <c r="J35" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -1892,7 +1956,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>TRIPLE 4X1 (nueva)</t>
+          <t>TRIPLE · 4X1</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -1906,11 +1970,7 @@
       <c r="G36" s="11" t="n"/>
       <c r="H36" s="13" t="n"/>
       <c r="I36" s="11" t="n"/>
-      <c r="J36" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -1928,9 +1988,9 @@
           <t>Abono Plantilla</t>
         </is>
       </c>
-      <c r="D37" s="14" t="inlineStr">
-        <is>
-          <t>FERTILIZACION PLANTILLA (nueva)</t>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>FERTILIZACION · PLANTILLA</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
@@ -1944,11 +2004,7 @@
       <c r="G37" s="11" t="n"/>
       <c r="H37" s="13" t="n"/>
       <c r="I37" s="11" t="n"/>
-      <c r="J37" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -1968,7 +2024,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>FERTILIZACION 2X1 (nueva)</t>
+          <t>FERTILIZACION · 2X1</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -1982,11 +2038,7 @@
       <c r="G38" s="11" t="n"/>
       <c r="H38" s="13" t="n"/>
       <c r="I38" s="11" t="n"/>
-      <c r="J38" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -2006,7 +2058,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>CULTIVO PLANTILLA (nueva)</t>
+          <t>CULTIVO · PLANTILLA</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -2020,11 +2072,7 @@
       <c r="G39" s="11" t="n"/>
       <c r="H39" s="13" t="n"/>
       <c r="I39" s="11" t="n"/>
-      <c r="J39" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -2044,7 +2092,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>CULTIVO 2X1 (nueva)</t>
+          <t>CULTIVO · 2X1</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -2058,11 +2106,7 @@
       <c r="G40" s="11" t="n"/>
       <c r="H40" s="13" t="n"/>
       <c r="I40" s="11" t="n"/>
-      <c r="J40" s="14" t="inlineStr">
-        <is>
-          <t>Labor nueva en la app, para que el supervisor escoja la variante al asignar</t>
-        </is>
-      </c>
+      <c r="J40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -2080,11 +2124,7 @@
           <t>Acequias</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>ACEQUIAS</t>
-        </is>
-      </c>
+      <c r="D41" s="11" t="n"/>
       <c r="E41" s="11" t="n"/>
       <c r="F41" s="12" t="n">
         <v>85000</v>
@@ -2407,7 +2447,7 @@
       <formula1>=Listas!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
-      <formula1>=Listas!$C$2:$C$20</formula1>
+      <formula1>=Listas!$C$2:$C$32</formula1>
     </dataValidation>
     <dataValidation sqref="E5:E66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
       <formula1>=Listas!$D$2:$D$5</formula1>
@@ -5180,7 +5220,7 @@
       <formula1>=Listas!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
-      <formula1>=Listas!$C$2:$C$20</formula1>
+      <formula1>=Listas!$C$2:$C$32</formula1>
     </dataValidation>
     <dataValidation sqref="N5:N54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
       <formula1>=Listas!$D$2:$D$5</formula1>
@@ -28832,17 +28872,17 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>FERTILIZACION</t>
+          <t>MODALIDADES (ya en la app)</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>El abono tiene 3 precios (plantilla, 2x1, 4x1). ¿Cómo se sabe cuál es?</t>
+          <t>Desde el 2-oct la app pide la modalidad al asignar: DESPEJE 0x0 / 2x1 mecanizada / 4x1 quemada · REENCALLE sencillo / 2x1 / verde · SUBSUELO y TRIPLE plantilla / 2x1 / 4x1 · ACEQUIAS 1 / 2 / 3 pases. ¿Está completa y bien escrita?</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Crear 3 labores en la app y que el supervisor escoja al asignar</t>
+          <t>Sí, así quedó (se puede cambiar en Más → Listas sin publicar)</t>
         </is>
       </c>
       <c r="D5" s="11" t="n"/>
@@ -28851,17 +28891,17 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>SUBSUELO / TRIPLE</t>
+          <t>TRIPLE</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Para proveedores hay «normal» y «4x1». ¿Cómo se sabe cuál es?</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Crear SUBSUELO 4X1 y TRIPLE 4X1 y que el supervisor escoja</t>
+          <t>En la hoja escrita el triple quedó con la llave vacía. ¿Tiene las mismas modalidades del subsuelo (plantilla, 2x1, 4x1)?</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Las mismas del subsuelo</t>
         </is>
       </c>
       <c r="D6" s="11" t="n"/>
@@ -28870,17 +28910,17 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>CULTIVO</t>
+          <t>FERTILIZACION</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Cultivo aporque: plantilla o 2x1 (proveedores). ¿Cómo se sabe?</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>Crear CULTIVO PLANTILLA y CULTIVO 2X1 y que el supervisor escoja</t>
+          <t>La hoja la deja SIN modalidad, pero la tabla de precios trae Abono plantilla, 2x1 y 4x1. ¿Se le ponen esas tres modalidades?</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Sí: plantilla / 2x1 / 4x1</t>
         </is>
       </c>
       <c r="D7" s="11" t="n"/>
@@ -28889,17 +28929,17 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>REENCALLE V</t>
+          <t>CULTIVO</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>¿La «REENCALLE V» de la app es el «Reencalle caña cruda / caña verde» de la tabla?</t>
+          <t>La tabla trae Cultivo aporque plantilla y 2x1 (proveedores). ¿Se le ponen esas modalidades?</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Sí: se cobra con ese precio</t>
+          <t>Sí: plantilla / 2x1</t>
         </is>
       </c>
       <c r="D8" s="11" t="n"/>
@@ -28908,17 +28948,17 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>ACEQUIAS</t>
+          <t>DESPEJE 2X1</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>¿Se cobra por hectárea o por hectómetro? En la app hay registros de las dos formas.</t>
+          <t>«2x1 verde limpio»: ¿el 2x1 mecanizado es siempre caña verde y limpia? ¿Hay un 2x1 quemado?</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Por hectómetro (es longitud de zanja)</t>
+          <t>2x1 = mecanizada en verde; 4x1 = quemada</t>
         </is>
       </c>
       <c r="D9" s="11" t="n"/>
@@ -28927,17 +28967,17 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>DESPEJE 0 X 0</t>
+          <t>ACEQUIAS</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>¿Qué es y qué precio tiene? (≈109 ha registradas en Pichichí, Riopaila, Risaralda y San Carlos)</t>
+          <t>¿El precio es por PASE (1, 2 o 3) o por hectómetro? ¿Un 2 pases cuesta el doble de uno?</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Mismo precio que Despeje, salvo que digan otro</t>
+          <t>Precio por modalidad (1, 2 o 3 pases)</t>
         </is>
       </c>
       <c r="D10" s="11" t="n"/>
@@ -28989,12 +29029,12 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Las ~4.750 labores desde mayo no tienen variante. ¿Qué precio toman?</t>
+          <t>Lo registrado antes del 2-oct no tiene modalidad. ¿Qué modalidad se les pone?</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>El de la variante más común; se puede corregir línea por línea antes de facturar</t>
+          <t>Administración la completa en lote en Facturación (filtro «Sin modalidad»)</t>
         </is>
       </c>
       <c r="D13" s="11" t="n"/>
@@ -29284,7 +29324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29342,7 +29382,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DESPEJE</t>
+          <t>DESPEJE · TODAS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -29384,7 +29424,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DESPEJE 0 X 0</t>
+          <t>DESPEJE · 0X0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -29421,7 +29461,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>REENCALLE</t>
+          <t>DESPEJE · 2X1 MECANIZADA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -29453,7 +29493,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>REENCALLE V</t>
+          <t>DESPEJE · 4X1 QUEMADA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -29475,7 +29515,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TRIPLE</t>
+          <t>REENCALLE · TODAS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -29492,7 +29532,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TRIPLE 4X1 (nueva)</t>
+          <t>REENCALLE · SENCILLO</t>
         </is>
       </c>
     </row>
@@ -29504,7 +29544,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SUBSUELO</t>
+          <t>REENCALLE · 2X1</t>
         </is>
       </c>
     </row>
@@ -29516,7 +29556,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SUBSUELO 4X1 (nueva)</t>
+          <t>REENCALLE · VERDE</t>
         </is>
       </c>
     </row>
@@ -29528,7 +29568,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FERTILIZACION PLANTILLA (nueva)</t>
+          <t>SUBSUELO · TODAS</t>
         </is>
       </c>
     </row>
@@ -29540,7 +29580,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FERTILIZACION 2X1 (nueva)</t>
+          <t>SUBSUELO · PLANTILLA</t>
         </is>
       </c>
     </row>
@@ -29552,61 +29592,145 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FERTILIZACION 4X1 (nueva)</t>
+          <t>SUBSUELO · 2X1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="C13" t="inlineStr">
         <is>
-          <t>CULTIVO</t>
+          <t>SUBSUELO · 4X1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="C14" t="inlineStr">
         <is>
-          <t>CULTIVO PLANTILLA (nueva)</t>
+          <t>TRIPLE · TODAS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="C15" t="inlineStr">
         <is>
-          <t>CULTIVO 2X1 (nueva)</t>
+          <t>TRIPLE · PLANTILLA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
         <is>
-          <t>ACEQUIAS</t>
+          <t>TRIPLE · 2X1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="C17" t="inlineStr">
         <is>
-          <t>DEVOLUCIÓN DE BASURA</t>
+          <t>TRIPLE · 4X1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="C18" t="inlineStr">
         <is>
-          <t>OFICIOS VARIOS (hora)</t>
+          <t>FERTILIZACION · TODAS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="C19" t="inlineStr">
         <is>
-          <t>OFICIOS VARIOS JORNAL (nueva)</t>
+          <t>FERTILIZACION · PLANTILLA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="C20" t="inlineStr">
+        <is>
+          <t>FERTILIZACION · 2X1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FERTILIZACION · 4X1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CULTIVO · TODAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CULTIVO · PLANTILLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CULTIVO · 2X1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · 1 PASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · 2 PASES</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · 3 PASES</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · POR HECTÓMETRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DEVOLUCIÓN DE BASURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OFICIOS VARIOS (hora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>OFICIOS VARIOS (jornal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Otra (ver observación)</t>
         </is>

</xml_diff>

<commit_message>
docs(facturación): modalidad desde el operario, sugerida 2x1 / 2 pases y regla de acequias
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
+++ b/facturacion/ASM_solicitud_tarifas_facturacion.xlsx
@@ -1248,7 +1248,11 @@
           <t>Acequias</t>
         </is>
       </c>
-      <c r="D17" s="11" t="n"/>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · HECTÓMETRO (incluye hasta 2 pases)</t>
+        </is>
+      </c>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="12" t="n">
         <v>70000</v>
@@ -2124,7 +2128,11 @@
           <t>Acequias</t>
         </is>
       </c>
-      <c r="D41" s="11" t="n"/>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>ACEQUIAS · HECTÓMETRO (incluye hasta 2 pases)</t>
+        </is>
+      </c>
       <c r="E41" s="11" t="n"/>
       <c r="F41" s="12" t="n">
         <v>85000</v>
@@ -2447,7 +2455,7 @@
       <formula1>=Listas!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
-      <formula1>=Listas!$C$2:$C$32</formula1>
+      <formula1>=Listas!$C$2:$C$30</formula1>
     </dataValidation>
     <dataValidation sqref="E5:E66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
       <formula1>=Listas!$D$2:$D$5</formula1>
@@ -5220,7 +5228,7 @@
       <formula1>=Listas!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
-      <formula1>=Listas!$C$2:$C$32</formula1>
+      <formula1>=Listas!$C$2:$C$30</formula1>
     </dataValidation>
     <dataValidation sqref="N5:N54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Escoja un valor de la lista." type="list">
       <formula1>=Listas!$D$2:$D$5</formula1>
@@ -28877,7 +28885,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Desde el 2-oct la app pide la modalidad al asignar: DESPEJE 0x0 / 2x1 mecanizada / 4x1 quemada · REENCALLE sencillo / 2x1 / verde · SUBSUELO y TRIPLE plantilla / 2x1 / 4x1 · ACEQUIAS 1 / 2 / 3 pases. ¿Está completa y bien escrita?</t>
+          <t>Desde el 2-oct la app pide la modalidad al asignar: DESPEJE 0x0 / 2x1 mecanizada / 4x1 quemada · REENCALLE sencillo / 2x1 / verde · SUBSUELO y TRIPLE plantilla / 2x1 / 4x1 · ACEQUIAS 1 / 2 / 3 pases. De entrada TODO viene en 2X1 y las acequias en 2 PASES; el operario la confirma al cerrar. ¿Está completa?</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
@@ -28972,12 +28980,12 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>¿El precio es por PASE (1, 2 o 3) o por hectómetro? ¿Un 2 pases cuesta el doble de uno?</t>
+          <t>Regla del 2-oct: el hectómetro pagado incluye hasta 2 pases; desde el 3.º cada pase es ADICIONAL. ¿Cuánto vale el pase adicional por hectómetro? ¿Igual al hectómetro?</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Precio por modalidad (1, 2 o 3 pases)</t>
+          <t>Mismo precio del hectómetro por cada pase adicional</t>
         </is>
       </c>
       <c r="D10" s="11" t="n"/>
@@ -29324,7 +29332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29683,54 +29691,40 @@
     <row r="25">
       <c r="C25" t="inlineStr">
         <is>
-          <t>ACEQUIAS · 1 PASE</t>
+          <t>ACEQUIAS · HECTÓMETRO (incluye hasta 2 pases)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" t="inlineStr">
         <is>
-          <t>ACEQUIAS · 2 PASES</t>
+          <t>ACEQUIAS · PASE ADICIONAL (3.º en adelante)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="C27" t="inlineStr">
         <is>
-          <t>ACEQUIAS · 3 PASES</t>
+          <t>DEVOLUCIÓN DE BASURA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="C28" t="inlineStr">
         <is>
-          <t>ACEQUIAS · POR HECTÓMETRO</t>
+          <t>OFICIOS VARIOS (hora)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="C29" t="inlineStr">
         <is>
-          <t>DEVOLUCIÓN DE BASURA</t>
+          <t>OFICIOS VARIOS (jornal)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="C30" t="inlineStr">
-        <is>
-          <t>OFICIOS VARIOS (hora)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>OFICIOS VARIOS (jornal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" t="inlineStr">
         <is>
           <t>Otra (ver observación)</t>
         </is>

</xml_diff>